<commit_message>
rename CW calcs and LF col
</commit_message>
<xml_diff>
--- a/data/LFData_WB_plus.xlsx
+++ b/data/LFData_WB_plus.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\seabr\Documents\Capstone\InRoomAirFilterScaleUp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9638511-E7B8-472A-96B5-942A24FA47E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AEFE0AA-3748-48BF-A525-43CB3493749D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4696" yWindow="3769" windowWidth="21637" windowHeight="13586" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-113" yWindow="-113" windowWidth="29076" windowHeight="18733" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="476">
   <si>
     <t>Country Name</t>
   </si>
@@ -1466,6 +1466,9 @@
   </si>
   <si>
     <t>chrome-extension://efaidnbmnnnibpcajpcglclefindmkaj/https://www.gov.im/media/1384637/isle-of-man-in-numbers-2024_compressed.pdf</t>
+  </si>
+  <si>
+    <t>Labour Force (2024)</t>
   </si>
 </sst>
 </file>
@@ -1798,6 +1801,7 @@
   <cols>
     <col min="1" max="1" width="25.109375" customWidth="1"/>
     <col min="4" max="4" width="26.44140625" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="14.4">
@@ -1813,8 +1817,8 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2">
-        <v>2024</v>
+      <c r="E1" s="2" t="s">
+        <v>475</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>4</v>

</xml_diff>